<commit_message>
Normaliza line endings, .gitattributes, actualiza reporte de gastos y crea reporte de debutantes de joyería
</commit_message>
<xml_diff>
--- a/Reporte_gastos/gastos desde 2025-05.xlsx
+++ b/Reporte_gastos/gastos desde 2025-05.xlsx
@@ -5,7 +5,7 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Reporte_gastos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Reporte_gastos\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -21,9 +21,9 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId4"/>
-    <pivotCache cacheId="2" r:id="rId5"/>
-    <pivotCache cacheId="15" r:id="rId6"/>
+    <pivotCache cacheId="2" r:id="rId4"/>
+    <pivotCache cacheId="3" r:id="rId5"/>
+    <pivotCache cacheId="4" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2040,109 +2040,7 @@
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -28471,7 +28369,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:AP16" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -28756,7 +28654,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica4" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A22:AZ35" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -29064,16 +28962,16 @@
     <dataField name="Suma de IMPORTE" fld="5" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="38">
+    <format dxfId="20">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="19">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="18">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="17">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="10">
@@ -29097,7 +28995,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="16">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29112,7 +29010,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="15">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29127,7 +29025,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29142,7 +29040,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="13">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29157,7 +29055,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="12">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29183,7 +29081,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:K16" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" defaultSubtotal="0">
@@ -29355,16 +29253,16 @@
     <dataField name="Suma de IMPORTE" fld="5" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="12">
-    <format dxfId="29">
+    <format dxfId="11">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="10">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="9">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="8">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29379,7 +29277,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="7">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29394,7 +29292,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="6">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29409,7 +29307,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="5">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29426,7 +29324,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="4">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29441,7 +29339,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="3">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29460,7 +29358,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="2">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="4">
@@ -29478,7 +29376,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="1">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">
@@ -29493,7 +29391,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="0">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="0" count="1">

</xml_diff>